<commit_message>
Sync HUL rating to HOLD/₹2,190; refresh Alphabet model
</commit_message>
<xml_diff>
--- a/assets/files/hul-business-model.xlsx
+++ b/assets/files/hul-business-model.xlsx
@@ -16,7 +16,16 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PE Valuation" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Football Field" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Cover'!$A$2:$K$39</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'IS'!$A$2:$G$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'BS'!$A$2:$G$58</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'CF'!$A$2:$G$47</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Key Ratios'!$A$2:$G$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'DCF Model'!$A$2:$K$80</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'PE Valuation'!$A$2:$K$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="7">'Football Field'!$A$2:$R$39</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
 </workbook>
 </file>
@@ -438,7 +447,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="242">
+  <cellXfs count="243">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -1160,6 +1169,9 @@
     </xf>
     <xf numFmtId="164" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="1" fontId="28" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1256,7 +1268,7 @@
                 <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>HUL Valuation Football Field  |  Current Price: ₹2,350</a:t>
+              <a:t>HUL Valuation Football Field  |  Current Price: ₹2,130</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1317,7 +1329,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1484,7 +1496,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1512,7 +1524,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1540,7 +1552,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1568,7 +1580,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1596,7 +1608,7 @@
                     </a:defRPr>
                   </a:pPr>
                   <a:r>
-                    <a:t/>
+                    <a:t>None</a:t>
                   </a:r>
                 </a:p>
               </txPr>
@@ -1622,7 +1634,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -1727,7 +1739,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1788,7 +1800,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1825,7 +1837,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -2079,7 +2091,7 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A2:K39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
@@ -2111,7 +2123,7 @@
     <row r="4" ht="24.75" customHeight="1" s="122">
       <c r="B4" s="127" t="inlineStr">
         <is>
-          <t>All figures in ₹ Millions (INR Mn) unless otherwise stated | Generated: 22 May 2026</t>
+          <t>All figures in ₹ Millions (INR Mn) unless otherwise stated | Updated: 14 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2254,7 @@
       </c>
       <c r="D22" s="140" t="inlineStr">
         <is>
-          <t>vs. ₹2,350</t>
+          <t>vs. ₹2,130</t>
         </is>
       </c>
       <c r="E22" s="140" t="inlineStr">
@@ -2322,7 +2334,7 @@
     <row r="30" ht="42" customHeight="1" s="122">
       <c r="B30" s="150" t="inlineStr">
         <is>
-          <t>The two valuation approaches diverge sharply: DCF implies ₹708 (‑70% downside); P/E implies ₹3,976 (+69% upside).</t>
+          <t>The two valuation approaches diverge sharply: DCF implies ₹712 (‑67% downside); P/E implies ₹2,826 (+33% upside).</t>
         </is>
       </c>
     </row>
@@ -2341,7 +2353,7 @@
       </c>
       <c r="C33" s="151" t="inlineStr">
         <is>
-          <t>DCF assumes 4.5% perpetual growth. Reverse DCF shows the market is pricing in ~9.3% — well above India's long-run nominal GDP and HUL's recent 6.5% 5Y CAGR.</t>
+          <t>DCF assumes 4.5% perpetual growth. Reverse DCF shows the market is pricing in ~9.1% — well above India's long-run nominal GDP and HUL's recent 6.5% 5Y CAGR.</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2392,7 @@
       </c>
       <c r="C37" s="151" t="inlineStr">
         <is>
-          <t>Use DCF as a discipline check, not a target. The implied 9.3% terminal growth is aggressive but not implausible for a dominant FMCG franchise in a fast-growing emerging economy. A blended view (e.g., 70% P/E weight, 30% DCF) gives a fair-value range of ₹2,500–₹3,200.</t>
+          <t>Use DCF as a discipline check, not a target. The implied ~9.1% terminal growth is aggressive for a mature FMCG franchise. A blended view (70% P/E, 30% DCF) gives a fair value of ~₹2,190 — essentially in line with the market price of ₹2,130. Rating: HOLD (no margin of safety at current levels; quality intact).</t>
         </is>
       </c>
     </row>
@@ -2426,8 +2438,8 @@
     <hyperlink ref="B12" location="'Key Ratios'!A1" display="Key Ratios"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
@@ -2437,9 +2449,9 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A2:G37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="121" min="1" max="1"/>
@@ -2840,7 +2852,7 @@
         <v>13220</v>
       </c>
       <c r="G26" s="162" t="n">
-        <v>49230</v>
+        <v>9570</v>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1" s="122">
@@ -2893,7 +2905,7 @@
         <v/>
       </c>
       <c r="G28" s="171">
-        <f>G27*0.17</f>
+        <f>G27*0.25</f>
         <v/>
       </c>
     </row>
@@ -2977,8 +2989,9 @@
       <c r="F33" s="173" t="n">
         <v>45.32</v>
       </c>
-      <c r="G33" s="173" t="n">
-        <v>64.01000000000001</v>
+      <c r="G33" s="173">
+        <f>G29/G35</f>
+        <v/>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1" s="122">
@@ -2999,8 +3012,9 @@
       <c r="F34" s="174" t="n">
         <v>45.32</v>
       </c>
-      <c r="G34" s="174" t="n">
-        <v>64.01000000000001</v>
+      <c r="G34" s="174">
+        <f>G29/G35</f>
+        <v/>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1" s="122">
@@ -3025,12 +3039,10 @@
         <f>F29/F33</f>
         <v/>
       </c>
-      <c r="G35" s="175">
-        <f>G29/G33</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36"/>
+      <c r="G35" s="175" t="n">
+        <v>2349.6</v>
+      </c>
+    </row>
     <row r="37" ht="13.5" customHeight="1" s="122">
       <c r="B37" s="137" t="inlineStr">
         <is>
@@ -3050,8 +3062,8 @@
     <mergeCell ref="B7:G7"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -3060,9 +3072,9 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A2:G58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="121" min="1" max="1"/>
@@ -3860,7 +3872,6 @@
         <v/>
       </c>
     </row>
-    <row r="57"/>
     <row r="58" ht="13.5" customHeight="1" s="122">
       <c r="B58" s="137" t="inlineStr">
         <is>
@@ -3882,8 +3893,8 @@
     <mergeCell ref="B7:G7"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -3892,9 +3903,9 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A2:G47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="121" min="1" max="1"/>
@@ -4543,7 +4554,6 @@
       <c r="F45" s="170" t="n"/>
       <c r="G45" s="170" t="n"/>
     </row>
-    <row r="46"/>
     <row r="47" ht="13.5" customHeight="1" s="122">
       <c r="B47" s="137" t="inlineStr">
         <is>
@@ -4564,8 +4574,8 @@
     <mergeCell ref="B7:G7"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -4574,9 +4584,9 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A2:G36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="121" min="1" max="1"/>
@@ -5209,7 +5219,6 @@
         <v/>
       </c>
     </row>
-    <row r="35"/>
     <row r="36" ht="13.5" customHeight="1" s="122">
       <c r="B36" s="137" t="inlineStr">
         <is>
@@ -5230,8 +5239,8 @@
     <mergeCell ref="B25:G25"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -5240,9 +5249,9 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K80"/>
+  <dimension ref="A2:K80"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="121" min="1" max="1"/>
@@ -5253,7 +5262,6 @@
     <col width="13" customWidth="1" style="121" min="9" max="11"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="45" customHeight="1" s="122">
       <c r="A2" s="123" t="n"/>
       <c r="B2" s="191" t="inlineStr">
@@ -5272,7 +5280,6 @@
     <row r="4" ht="30" customHeight="1" s="122">
       <c r="B4" s="193" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="122">
       <c r="B6" s="139" t="inlineStr">
         <is>
@@ -5388,11 +5395,10 @@
           <t>Current Share Price (₹)</t>
         </is>
       </c>
-      <c r="C17" s="197" t="n">
-        <v>2350</v>
-      </c>
-    </row>
-    <row r="18"/>
+      <c r="C17" s="242" t="n">
+        <v>2130</v>
+      </c>
+    </row>
     <row r="19" ht="15" customHeight="1" s="122">
       <c r="B19" s="146" t="inlineStr">
         <is>
@@ -5719,7 +5725,6 @@
         <v/>
       </c>
     </row>
-    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="122">
       <c r="B32" s="139" t="inlineStr">
         <is>
@@ -5803,7 +5808,6 @@
         <v/>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="122">
       <c r="B37" s="141" t="inlineStr">
         <is>
@@ -5826,7 +5830,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40" ht="15" customHeight="1" s="122">
       <c r="B40" s="139" t="inlineStr">
         <is>
@@ -5933,7 +5936,6 @@
         <v/>
       </c>
     </row>
-    <row r="50"/>
     <row r="51" ht="15" customHeight="1" s="122">
       <c r="B51" s="152" t="inlineStr">
         <is>
@@ -5956,8 +5958,6 @@
         <v/>
       </c>
     </row>
-    <row r="53"/>
-    <row r="54"/>
     <row r="55" ht="15.75" customHeight="1" s="122">
       <c r="B55" s="211" t="inlineStr">
         <is>
@@ -5972,7 +5972,6 @@
         </is>
       </c>
     </row>
-    <row r="57"/>
     <row r="58" ht="15" customHeight="1" s="122">
       <c r="B58" s="140" t="inlineStr">
         <is>
@@ -6272,8 +6271,8 @@
     <mergeCell ref="B2:K2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -6282,9 +6281,9 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A2:K37"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="121" min="1" max="1"/>
@@ -6295,7 +6294,6 @@
     <col width="13" customWidth="1" style="121" min="8" max="11"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="45" customHeight="1" s="122">
       <c r="A2" s="123" t="n"/>
       <c r="B2" s="191" t="inlineStr">
@@ -6314,7 +6312,6 @@
     <row r="4" ht="30" customHeight="1" s="122">
       <c r="B4" s="193" t="n"/>
     </row>
-    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="122">
       <c r="B6" s="139" t="inlineStr">
         <is>
@@ -6453,7 +6450,6 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
     <row r="13" ht="15" customHeight="1" s="122">
       <c r="B13" s="139" t="inlineStr">
         <is>
@@ -6516,7 +6512,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="122">
       <c r="B20" s="139" t="inlineStr">
         <is>
@@ -6556,7 +6551,6 @@
         <v/>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="15" customHeight="1" s="122">
       <c r="B25" s="139" t="inlineStr">
         <is>
@@ -6662,7 +6656,6 @@
         <v/>
       </c>
     </row>
-    <row r="31"/>
     <row r="32" ht="15" customHeight="1" s="122">
       <c r="B32" s="139" t="inlineStr">
         <is>
@@ -6703,7 +6696,6 @@
         <v/>
       </c>
     </row>
-    <row r="36"/>
     <row r="37" ht="15" customHeight="1" s="122">
       <c r="B37" s="231" t="inlineStr">
         <is>
@@ -6717,8 +6709,8 @@
     <mergeCell ref="B2:K2"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
 </file>
 
@@ -6727,9 +6719,9 @@
   <sheetPr filterMode="0">
     <tabColor rgb="FF1C39BB"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A2:H19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="10.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="46" customWidth="1" style="121" min="2" max="2"/>
@@ -6738,7 +6730,6 @@
     <col width="13" customWidth="1" style="121" min="6" max="8"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="18.75" customHeight="1" s="122">
       <c r="A2" s="123" t="n"/>
       <c r="B2" s="232" t="inlineStr">
@@ -6759,8 +6750,12 @@
           <t>Implied share price range by valuation methodology | Current price: ₹2,350</t>
         </is>
       </c>
-    </row>
-    <row r="4"/>
+      <c r="D3" s="121" t="inlineStr">
+        <is>
+          <t>Implied share price range by valuation methodology | Current price: ₹2,130</t>
+        </is>
+      </c>
+    </row>
     <row r="5" ht="15" customHeight="1" s="122">
       <c r="B5" s="139" t="inlineStr">
         <is>
@@ -6844,7 +6839,7 @@
         <v/>
       </c>
       <c r="H7" s="237" t="n">
-        <v>2350</v>
+        <v>2130</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="122">
@@ -6854,15 +6849,15 @@
         </is>
       </c>
       <c r="C8" s="142">
-        <f>('PE Valuation'!C17-'PE Valuation'!C18)*'PE Valuation'!C23</f>
+        <f>('PE Valuation'!C14-STDEV('PE Valuation'!C11:G11))*'PE Valuation'!C23</f>
         <v/>
       </c>
       <c r="D8" s="234">
-        <f>'PE Valuation'!C17*'PE Valuation'!C23</f>
+        <f>'PE Valuation'!C14*'PE Valuation'!C23</f>
         <v/>
       </c>
       <c r="E8" s="142">
-        <f>('PE Valuation'!C17+'PE Valuation'!C18)*'PE Valuation'!C23</f>
+        <f>('PE Valuation'!C14+STDEV('PE Valuation'!C11:G11))*'PE Valuation'!C23</f>
         <v/>
       </c>
       <c r="F8" s="235">
@@ -6910,13 +6905,13 @@
         </is>
       </c>
       <c r="C10" s="240" t="n">
-        <v>2150</v>
+        <v>2100</v>
       </c>
       <c r="D10" s="241" t="n">
         <v>2350</v>
       </c>
       <c r="E10" s="240" t="n">
-        <v>2680</v>
+        <v>2700</v>
       </c>
       <c r="F10" s="235">
         <f>E10-C10</f>
@@ -6928,9 +6923,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="122">
       <c r="B14" s="141" t="inlineStr">
         <is>
@@ -7025,8 +7017,8 @@
     </row>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>